<commit_message>
Add S2022 random-10 DRT workflows, tau-grid reporting, and outputs
</commit_message>
<xml_diff>
--- a/lambda_perturbation_result.xlsx
+++ b/lambda_perturbation_result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mitra\Downloads\matlab analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D79D3A-6B15-48D9-983B-01FF1ADCFABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA1A5CB-C6AD-42E7-A221-3DA031B22DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="50" activeTab="50" xr2:uid="{54EEB03B-E474-4362-ABD5-5443D823EEF5}"/>
   </bookViews>
@@ -7085,28 +7085,28 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>280.33999999999997</v>
+        <v>242.2</v>
       </c>
       <c r="B2">
-        <v>1E-4</v>
+        <v>0.1</v>
       </c>
       <c r="C2">
-        <v>67.083028629233141</v>
+        <v>113.753388492073</v>
       </c>
       <c r="D2">
-        <v>-1.5475239982848096E-2</v>
+        <v>-18.633758627701685</v>
       </c>
       <c r="E2">
-        <v>0.26845305433424982</v>
+        <v>41.741352574135156</v>
       </c>
       <c r="F2">
-        <v>0.26845305433424982</v>
+        <v>41.741352574135156</v>
       </c>
       <c r="G2">
-        <v>0.11934897733253454</v>
+        <v>58.024449111202259</v>
       </c>
       <c r="H2">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="I2">
         <v>3</v>
@@ -7405,16 +7405,16 @@
         <v>0.3</v>
       </c>
       <c r="B2">
-        <v>3.0000000000000001E-5</v>
+        <v>0.03</v>
       </c>
       <c r="C2">
-        <v>73.55633819321686</v>
+        <v>92.55685664962833</v>
       </c>
       <c r="D2">
-        <v>1518.2620771458937</v>
+        <v>1527.6155209372105</v>
       </c>
       <c r="E2">
-        <v>6.0146678046458089E-2</v>
+        <v>-18.633758627701685</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -7422,16 +7422,16 @@
         <v>0.5</v>
       </c>
       <c r="B3">
-        <v>5.0000000000000002E-5</v>
+        <v>0.05</v>
       </c>
       <c r="C3">
-        <v>73.529655426763583</v>
+        <v>100.20681716938664</v>
       </c>
       <c r="D3">
-        <v>1518.4028727611751</v>
+        <v>1529.8374653683991</v>
       </c>
       <c r="E3">
-        <v>2.3849581281285562E-2</v>
+        <v>-11.908718942144185</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -7439,16 +7439,16 @@
         <v>0.7</v>
       </c>
       <c r="B4">
-        <v>6.9999999999999994E-5</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="C4">
-        <v>73.527238181884897</v>
+        <v>106.16424617256973</v>
       </c>
       <c r="D4">
-        <v>1518.4700560765048</v>
+        <v>1531.462377004673</v>
       </c>
       <c r="E4">
-        <v>2.0561355099026412E-2</v>
+        <v>-6.6715747285472045</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -7456,13 +7456,13 @@
         <v>1</v>
       </c>
       <c r="B5">
-        <v>1E-4</v>
+        <v>0.1</v>
       </c>
       <c r="C5">
-        <v>73.512123093214868</v>
+        <v>113.753388492073</v>
       </c>
       <c r="D5">
-        <v>1518.5961063205477</v>
+        <v>1533.3410463484852</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -7473,16 +7473,16 @@
         <v>1.5</v>
       </c>
       <c r="B6">
-        <v>1.5000000000000001E-4</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="C6">
-        <v>73.503156809171657</v>
+        <v>125.3699453669919</v>
       </c>
       <c r="D6">
-        <v>1518.7345029817425</v>
+        <v>1535.7688831277887</v>
       </c>
       <c r="E6">
-        <v>-1.2197014133086284E-2</v>
+        <v>10.212053485974538</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -7490,16 +7490,16 @@
         <v>2</v>
       </c>
       <c r="B7">
-        <v>2.0000000000000001E-4</v>
+        <v>0.2</v>
       </c>
       <c r="C7">
-        <v>73.501600769729805</v>
+        <v>137.33396037359543</v>
       </c>
       <c r="D7">
-        <v>1518.8236282199273</v>
+        <v>1537.5984987668135</v>
       </c>
       <c r="E7">
-        <v>-1.4313725467730182E-2</v>
+        <v>20.729555571142978</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -7507,16 +7507,16 @@
         <v>3</v>
       </c>
       <c r="B8">
-        <v>3.0000000000000003E-4</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="C8">
-        <v>73.474392965155062</v>
+        <v>161.23559144757488</v>
       </c>
       <c r="D8">
-        <v>1519.0400744934484</v>
+        <v>1540.3585303842765</v>
       </c>
       <c r="E8">
-        <v>-5.1325042009688064E-2</v>
+        <v>41.741352574135156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>